<commit_message>
Prestentation et Conception du projet
</commit_message>
<xml_diff>
--- a/battery_cells_curated.xlsx
+++ b/battery_cells_curated.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X44"/>
+  <dimension ref="A1:X45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3545,6 +3545,42 @@
         <v>3</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Prismatic</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>101</v>
+      </c>
+      <c r="G45" t="n">
+        <v>221</v>
+      </c>
+      <c r="H45" t="n">
+        <v>155</v>
+      </c>
+      <c r="I45" t="n">
+        <v>2150</v>
+      </c>
+      <c r="J45" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="K45" t="n">
+        <v>99</v>
+      </c>
+      <c r="L45" t="n">
+        <v>180</v>
+      </c>
+      <c r="W45" t="n">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>